<commit_message>
correcciones varias semantico soporte de cadenas, arreglos en automatas, correcciones en ciclos
</commit_message>
<xml_diff>
--- a/src/data/TAS.xlsx
+++ b/src/data/TAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matem\Documents\Proyecto Sintaxis Node\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF9648C-370C-49BD-B0E1-BE728D220711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAB00A8-F5D4-488B-BD8D-0915573A0DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="118">
   <si>
     <t>Program</t>
   </si>
@@ -824,14 +824,23 @@
     <t xml:space="preserve">For </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">for ( </t>
+    <t>Condicion</t>
+  </si>
+  <si>
+    <t>TerminoLogico CondicionPrima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CondicionPrima </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>|</t>
     </r>
     <r>
       <rPr>
@@ -841,16 +850,27 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">Asignacion </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">; </t>
+      <t xml:space="preserve"> TerminoLogico CondicionPrima</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">TerminoLogico </t>
+  </si>
+  <si>
+    <t>FactorLogico TerminoLogicoPrima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TerminoLogicoPrima </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">&amp; </t>
     </r>
     <r>
       <rPr>
@@ -860,17 +880,13 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">Condicion </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">) { </t>
-    </r>
+      <t>FactorLogico TerminoLogicoPrima </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">FactorLogico </t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -879,6 +895,255 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
+      <t xml:space="preserve">ExpArit </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">opRel </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>ExpArit</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">! </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>FactorLogico</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">ExpArit </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">opRel </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>ExpArit</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">ExpArit </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">opRel </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>ExpArit</t>
+    </r>
+  </si>
+  <si>
+    <t>cteCadena</t>
+  </si>
+  <si>
+    <t>[ cteReal ]</t>
+  </si>
+  <si>
+    <t>Leer ;</t>
+  </si>
+  <si>
+    <t>{ Condicion }</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Program </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">id ; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>DeclaracionVar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> {</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Secuencia </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>}</t>
+    </r>
+  </si>
+  <si>
+    <t>cteReal</t>
+  </si>
+  <si>
+    <t>ExpArit</t>
+  </si>
+  <si>
+    <r>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>, ExpArit ListaElementosPrim</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>a</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Asignacion :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">ExpArit </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">{ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
       <t xml:space="preserve">Secuencia </t>
     </r>
     <r>
@@ -892,275 +1157,7 @@
     </r>
   </si>
   <si>
-    <t>Condicion</t>
-  </si>
-  <si>
-    <t>TerminoLogico CondicionPrima</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CondicionPrima </t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>|</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> TerminoLogico CondicionPrima</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">TerminoLogico </t>
-  </si>
-  <si>
-    <t>FactorLogico TerminoLogicoPrima</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TerminoLogicoPrima </t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">&amp; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>FactorLogico TerminoLogicoPrima </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">FactorLogico </t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">ExpArit </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">opRel </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>ExpArit</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">! </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>FactorLogico</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">ExpArit </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">opRel </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>ExpArit</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">ExpArit </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">opRel </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>ExpArit</t>
-    </r>
-  </si>
-  <si>
-    <t>cteCadena</t>
-  </si>
-  <si>
-    <t>[ cteReal ]</t>
-  </si>
-  <si>
-    <t>Leer ;</t>
-  </si>
-  <si>
-    <t>{ Condicion }</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Program </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">id ; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>DeclaracionVar</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> {</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Secuencia </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>}</t>
-    </r>
-  </si>
-  <si>
-    <t>cteReal</t>
-  </si>
-  <si>
-    <t>ExpArit</t>
-  </si>
-  <si>
-    <r>
-      <t> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>, ExpArit ListaElementosPrim</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>a</t>
-    </r>
+    <t>:</t>
   </si>
 </sst>
 </file>
@@ -1420,7 +1417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1470,6 +1467,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1685,7 +1683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG998"/>
+  <dimension ref="A1:AH998"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" customWidth="1"/>
@@ -1721,7 +1719,7 @@
     <col min="33" max="33" width="16.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1805,7 +1803,7 @@
         <v>26</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="AD1" s="2" t="s">
         <v>27</v>
@@ -1817,15 +1815,18 @@
         <v>29</v>
       </c>
       <c r="AG1" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
+      </c>
+      <c r="AH1" s="39" t="s">
+        <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -1858,7 +1859,7 @@
       <c r="AE2" s="9"/>
       <c r="AF2" s="10"/>
     </row>
-    <row r="3" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
         <v>31</v>
       </c>
@@ -1898,7 +1899,7 @@
       <c r="AE3" s="15"/>
       <c r="AF3" s="14"/>
     </row>
-    <row r="4" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>34</v>
       </c>
@@ -1936,7 +1937,7 @@
       <c r="AE4" s="15"/>
       <c r="AF4" s="14"/>
     </row>
-    <row r="5" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>36</v>
       </c>
@@ -1974,7 +1975,7 @@
       <c r="AE5" s="15"/>
       <c r="AF5" s="14"/>
     </row>
-    <row r="6" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>38</v>
       </c>
@@ -2010,11 +2011,11 @@
       <c r="AC6" s="15"/>
       <c r="AD6" s="14"/>
       <c r="AE6" s="17" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AF6" s="14"/>
     </row>
-    <row r="7" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>40</v>
       </c>
@@ -2062,7 +2063,7 @@
       <c r="AE7" s="15"/>
       <c r="AF7" s="14"/>
     </row>
-    <row r="8" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
         <v>42</v>
       </c>
@@ -2076,7 +2077,7 @@
       <c r="G8" s="12"/>
       <c r="H8" s="12"/>
       <c r="I8" s="34" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J8" s="13" t="s">
         <v>44</v>
@@ -2110,7 +2111,7 @@
       <c r="AE8" s="15"/>
       <c r="AF8" s="14"/>
     </row>
-    <row r="9" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>48</v>
       </c>
@@ -2150,7 +2151,7 @@
       <c r="AE9" s="15"/>
       <c r="AF9" s="14"/>
     </row>
-    <row r="10" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>50</v>
       </c>
@@ -2188,7 +2189,7 @@
       <c r="AE10" s="15"/>
       <c r="AF10" s="14"/>
     </row>
-    <row r="11" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
         <v>52</v>
       </c>
@@ -2256,7 +2257,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
         <v>54</v>
       </c>
@@ -2293,17 +2294,19 @@
       <c r="Z12" s="12"/>
       <c r="AA12" s="14"/>
       <c r="AB12" s="14"/>
-      <c r="AC12" s="15"/>
+      <c r="AC12" s="15" t="s">
+        <v>108</v>
+      </c>
       <c r="AD12" s="14"/>
       <c r="AE12" s="23" t="s">
         <v>55</v>
       </c>
       <c r="AF12" s="14"/>
       <c r="AG12" s="37" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
         <v>55</v>
       </c>
@@ -2350,7 +2353,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:34" ht="13.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
         <v>58</v>
       </c>
@@ -2409,8 +2412,11 @@
       <c r="AF14" s="16" t="s">
         <v>39</v>
       </c>
+      <c r="AH14" s="14" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="15" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">
         <v>61</v>
       </c>
@@ -2457,7 +2463,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="11" t="s">
         <v>63</v>
       </c>
@@ -2468,7 +2474,9 @@
       </c>
       <c r="E16" s="12"/>
       <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
+      <c r="G16" s="14" t="s">
+        <v>39</v>
+      </c>
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
       <c r="J16" s="12"/>
@@ -2518,8 +2526,11 @@
       <c r="AF16" s="16" t="s">
         <v>39</v>
       </c>
+      <c r="AH16" s="14" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="17" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="11" t="s">
         <v>66</v>
       </c>
@@ -2566,7 +2577,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="11" t="s">
         <v>68</v>
       </c>
@@ -2577,7 +2588,9 @@
       </c>
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
+      <c r="G18" s="14" t="s">
+        <v>39</v>
+      </c>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
       <c r="J18" s="12"/>
@@ -2629,8 +2642,11 @@
       <c r="AF18" s="16" t="s">
         <v>39</v>
       </c>
+      <c r="AH18" s="14" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="19" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="11" t="s">
         <v>70</v>
       </c>
@@ -2674,10 +2690,10 @@
       </c>
       <c r="AF19" s="14"/>
       <c r="AG19" s="37" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="11" t="s">
         <v>74</v>
       </c>
@@ -2715,7 +2731,7 @@
       </c>
       <c r="AF20" s="14"/>
     </row>
-    <row r="21" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="11" t="s">
         <v>76</v>
       </c>
@@ -2762,7 +2778,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:33" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:34" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="26" t="s">
         <v>78</v>
       </c>
@@ -2791,7 +2807,7 @@
       <c r="X22" s="12"/>
       <c r="Y22" s="12"/>
       <c r="Z22" s="21" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AA22" s="14"/>
       <c r="AB22" s="14"/>
@@ -2802,7 +2818,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
         <v>79</v>
       </c>
@@ -2840,7 +2856,7 @@
       <c r="AE23" s="15"/>
       <c r="AF23" s="14"/>
     </row>
-    <row r="24" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>81</v>
       </c>
@@ -2878,7 +2894,7 @@
       <c r="AE24" s="15"/>
       <c r="AF24" s="14"/>
     </row>
-    <row r="25" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>83</v>
       </c>
@@ -2924,7 +2940,7 @@
       </c>
       <c r="AF25" s="14"/>
     </row>
-    <row r="26" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>86</v>
       </c>
@@ -2964,7 +2980,7 @@
       <c r="AE26" s="15"/>
       <c r="AF26" s="14"/>
     </row>
-    <row r="27" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
         <v>88</v>
       </c>
@@ -3002,7 +3018,7 @@
       <c r="AE27" s="15"/>
       <c r="AF27" s="14"/>
     </row>
-    <row r="28" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>90</v>
       </c>
@@ -3042,7 +3058,7 @@
       <c r="AE28" s="15"/>
       <c r="AF28" s="14"/>
     </row>
-    <row r="29" spans="1:33" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:34" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
         <v>92</v>
       </c>
@@ -3080,7 +3096,7 @@
       <c r="AE29" s="15"/>
       <c r="AF29" s="14"/>
     </row>
-    <row r="30" spans="1:33" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:34" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
         <v>94</v>
       </c>
@@ -3101,7 +3117,7 @@
       <c r="P30" s="12"/>
       <c r="Q30" s="12"/>
       <c r="R30" s="16" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="S30" s="12"/>
       <c r="T30" s="12"/>
@@ -3118,13 +3134,13 @@
       <c r="AE30" s="15"/>
       <c r="AF30" s="14"/>
     </row>
-    <row r="31" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D31" s="12"/>
       <c r="E31" s="13"/>
@@ -3135,7 +3151,7 @@
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
       <c r="L31" s="13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M31" s="12"/>
       <c r="N31" s="12"/>
@@ -3144,11 +3160,11 @@
       <c r="Q31" s="12"/>
       <c r="R31" s="12"/>
       <c r="S31" s="13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="T31" s="12"/>
       <c r="U31" s="13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="V31" s="12"/>
       <c r="W31" s="12"/>
@@ -3160,11 +3176,11 @@
       <c r="AC31" s="15"/>
       <c r="AD31" s="14"/>
       <c r="AE31" s="25" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AF31" s="14"/>
     </row>
-    <row r="32" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
         <v>36</v>
       </c>
@@ -3202,7 +3218,7 @@
     </row>
     <row r="33" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B33" s="12"/>
       <c r="C33" s="12"/>
@@ -3239,7 +3255,7 @@
       <c r="Z33" s="12"/>
       <c r="AA33" s="14"/>
       <c r="AB33" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AC33" s="15"/>
       <c r="AD33" s="14"/>
@@ -3248,11 +3264,11 @@
     </row>
     <row r="34" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B34" s="12"/>
       <c r="C34" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="13"/>
@@ -3263,7 +3279,7 @@
       <c r="J34" s="12"/>
       <c r="K34" s="12"/>
       <c r="L34" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M34" s="12"/>
       <c r="N34" s="12"/>
@@ -3272,7 +3288,7 @@
       <c r="Q34" s="12"/>
       <c r="R34" s="12"/>
       <c r="S34" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="T34" s="12"/>
       <c r="U34" s="12"/>
@@ -3281,20 +3297,20 @@
       <c r="X34" s="12"/>
       <c r="Y34" s="12"/>
       <c r="Z34" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AA34" s="14"/>
       <c r="AB34" s="14"/>
       <c r="AC34" s="15"/>
       <c r="AD34" s="14"/>
       <c r="AE34" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AF34" s="14"/>
     </row>
     <row r="35" spans="1:32" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B35" s="12"/>
       <c r="C35" s="12"/>
@@ -3330,7 +3346,7 @@
       <c r="Y35" s="12"/>
       <c r="Z35" s="12"/>
       <c r="AA35" s="19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AB35" s="16" t="s">
         <v>39</v>
@@ -3342,17 +3358,17 @@
     </row>
     <row r="36" spans="1:32" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B36" s="28"/>
       <c r="C36" s="29" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D36" s="28"/>
       <c r="E36" s="29"/>
       <c r="F36" s="28"/>
       <c r="G36" s="34" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H36" s="28"/>
       <c r="I36" s="28"/>
@@ -3366,11 +3382,11 @@
       <c r="Q36" s="28"/>
       <c r="R36" s="28"/>
       <c r="S36" s="30" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="T36" s="28"/>
       <c r="U36" s="29" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="V36" s="28"/>
       <c r="W36" s="28"/>
@@ -3382,7 +3398,7 @@
       <c r="AC36" s="32"/>
       <c r="AD36" s="31"/>
       <c r="AE36" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AF36" s="31"/>
     </row>
@@ -4352,6 +4368,6 @@
     <row r="998" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>